<commit_message>
Adição de novos itens no dicionario
</commit_message>
<xml_diff>
--- a/docs/modelo_dicionario_de_dados.xlsx
+++ b/docs/modelo_dicionario_de_dados.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="134">
   <si>
     <t xml:space="preserve">MODELO DE DICIONÁRIO DE DADOS</t>
   </si>
@@ -105,162 +105,284 @@
     <t xml:space="preserve">Campo do nome do funcionario</t>
   </si>
   <si>
-    <t xml:space="preserve">id_status</t>
+    <t xml:space="preserve">status</t>
   </si>
   <si>
     <t xml:space="preserve">FK</t>
   </si>
   <si>
-    <t xml:space="preserve">Campo qual status é vinculado</t>
+    <t xml:space="preserve">Cadastro do Status do funcionario</t>
   </si>
   <si>
     <t xml:space="preserve">id_cargo</t>
   </si>
   <si>
+    <t xml:space="preserve">UNIQUE(id, id_cargo)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cargo qual funcionario é vinculado</t>
   </si>
   <si>
-    <t xml:space="preserve">criacao</t>
+    <t xml:space="preserve">data_cadastro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Primaria de Indentificação do cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do nome do cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e-mail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email do cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cadastro do Status do cliente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_funcionario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_funcionario_cargo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave Primaria de Indentificação do equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo do nome do equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_cliente </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave estrangeira id do cliente dono do equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_marca</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">Chave estrangeira do id </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">marca do equipamento</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">id_modelo</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">Chave estrangeira do id </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Modelo do Equipamento</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">id_tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave estrangeira do id tipo de equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Numero de Serie do equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">imei</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cadastro do Status do equipamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cargo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_cargo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNIQUE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DATETIME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">marca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chave primaria de Indentificação da Marca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_marca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">modelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_modelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INSTRUÇÕES E EXEMPLO PRÁTICO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como preencher o Dicionário de Dados e Exemplo Demonstrativo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Nome da Tabela:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Identificador da tabela em minúsculas/snake_case (ex: alunos, cursos).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Nome do Campo:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nome exato da coluna no banco de dados (ex: id_aluno, cpf, data_nascimento).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Tipo de Dado:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo do atributo no SGBD (ex: INT, VARCHAR, DECIMAL, DATE). Use a lista suspensa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Tamanho / Precisão:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tamanho do campo, se aplicável (ex: 100 para VARCHAR, 10,2 para DECIMAL).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Chave (PK/FK):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Informe se o campo é Chave Primária (PK), Chave Estrangeira (FK), ou Ambos (PFK).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Permite Nulo?:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Selecione SIM se aceitar valores nulos (NULL) ou NÃO se for NOT NULL.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7. Valor Padrão:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor atribuído automaticamente caso nenhum seja informado (ex: CURRENT_TIMESTAMP, 0, 'ATIVO').</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8. Tabela Referenciada:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caso seja FK, informe a tabela e campo de origem (ex: cursos(id_curso)).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9. Descrição / Regra:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Explicação clara do significado do dado e eventuais restrições ou regras de negócio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exemplo Preenchido:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nome do Campo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor Padrão</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tabela / Campo Referenciado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tb_alunos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_aluno</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUTO_INCREMENT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Identificador único do aluno.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_completo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VARCHAR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nenhum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nome civil completo do aluno.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cpf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apenas números. Deve ser único (UNIQUE).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data_nascimento</t>
   </si>
   <si>
     <t xml:space="preserve">DATE</t>
   </si>
   <si>
-    <t xml:space="preserve">Campo de data de criação do funcionario</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cliente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chave Primaria de Indentificação do cliente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo do nome do cliente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">equipamento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chave Primaria de Indentificação do equipamento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Campo do nome do equipamento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INSTRUÇÕES E EXEMPLO PRÁTICO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como preencher o Dicionário de Dados e Exemplo Demonstrativo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Nome da Tabela:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Identificador da tabela em minúsculas/snake_case (ex: alunos, cursos).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Nome do Campo:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nome exato da coluna no banco de dados (ex: id_aluno, cpf, data_nascimento).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Tipo de Dado:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tipo do atributo no SGBD (ex: INT, VARCHAR, DECIMAL, DATE). Use a lista suspensa.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Tamanho / Precisão:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tamanho do campo, se aplicável (ex: 100 para VARCHAR, 10,2 para DECIMAL).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. Chave (PK/FK):</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Informe se o campo é Chave Primária (PK), Chave Estrangeira (FK), ou Ambos (PFK).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6. Permite Nulo?:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Selecione SIM se aceitar valores nulos (NULL) ou NÃO se for NOT NULL.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7. Valor Padrão:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valor atribuído automaticamente caso nenhum seja informado (ex: CURRENT_TIMESTAMP, 0, 'ATIVO').</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8. Tabela Referenciada:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Caso seja FK, informe a tabela e campo de origem (ex: cursos(id_curso)).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9. Descrição / Regra:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Explicação clara do significado do dado e eventuais restrições ou regras de negócio.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exemplo Preenchido:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nome do Campo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valor Padrão</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tabela / Campo Referenciado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tb_alunos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id_aluno</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUTO_INCREMENT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Identificador único do aluno.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nome_completo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VARCHAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nenhum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nome civil completo do aluno.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cpf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Apenas números. Deve ser único (UNIQUE).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">data_nascimento</t>
-  </si>
-  <si>
     <t xml:space="preserve">Data de nascimento para cálculo de idade.</t>
   </si>
   <si>
@@ -328,9 +450,6 @@
   </si>
   <si>
     <t xml:space="preserve">DECIMAL(10,2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DATETIME</t>
   </si>
   <si>
     <t xml:space="preserve">BOOLEAN</t>
@@ -346,7 +465,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -415,11 +534,6 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Consolas"/>
       <family val="0"/>
     </font>
     <font>
@@ -500,7 +614,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -541,7 +655,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -561,15 +675,19 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -581,7 +699,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -837,7 +955,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I1048576"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr defaultColWidth="8.34375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
@@ -980,9 +1098,11 @@
       <c r="F12" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="G12" s="8"/>
+      <c r="G12" s="8" t="n">
+        <v>1</v>
+      </c>
       <c r="H12" s="7"/>
-      <c r="I12" s="15" t="s">
+      <c r="I12" s="10" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1003,599 +1123,953 @@
       <c r="F13" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="G13" s="8"/>
+      <c r="G13" s="8" t="s">
+        <v>31</v>
+      </c>
       <c r="H13" s="7"/>
-      <c r="I13" s="15" t="s">
-        <v>31</v>
+      <c r="I13" s="10" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="C14" s="16" t="s">
+      <c r="B14" s="11" t="s">
         <v>33</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>25</v>
       </c>
       <c r="D14" s="0"/>
       <c r="E14" s="0"/>
-      <c r="F14" s="16" t="s">
+      <c r="F14" s="15" t="s">
         <v>21</v>
       </c>
       <c r="G14" s="0"/>
       <c r="H14" s="0"/>
-      <c r="I14" s="0" t="s">
+      <c r="I14" s="14"/>
+    </row>
+    <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="7"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="10"/>
+    </row>
+    <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0"/>
-      <c r="B15" s="0"/>
-      <c r="C15" s="0"/>
-      <c r="D15" s="0"/>
-      <c r="E15" s="0"/>
-      <c r="F15" s="0"/>
-      <c r="G15" s="0"/>
-      <c r="H15" s="0"/>
-      <c r="I15" s="0"/>
-    </row>
-    <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0"/>
-      <c r="B16" s="0"/>
-      <c r="C16" s="0"/>
-      <c r="D16" s="0"/>
-      <c r="E16" s="0"/>
-      <c r="F16" s="0"/>
-      <c r="G16" s="0"/>
-      <c r="H16" s="0"/>
-      <c r="I16" s="0"/>
+      <c r="B16" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H16" s="7"/>
+      <c r="I16" s="10" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0"/>
-      <c r="B17" s="0"/>
-      <c r="C17" s="0"/>
-      <c r="D17" s="0"/>
-      <c r="E17" s="0"/>
-      <c r="F17" s="0"/>
-      <c r="G17" s="0"/>
-      <c r="H17" s="0"/>
-      <c r="I17" s="0"/>
+      <c r="A17" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G17" s="12"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="14" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0"/>
-      <c r="B18" s="0"/>
-      <c r="C18" s="0"/>
-      <c r="D18" s="0"/>
-      <c r="E18" s="0"/>
-      <c r="F18" s="0"/>
-      <c r="G18" s="0"/>
-      <c r="H18" s="0"/>
-      <c r="I18" s="0"/>
+      <c r="A18" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" s="12"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="14" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7"/>
-      <c r="B19" s="7"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="7"/>
-      <c r="I19" s="15"/>
+      <c r="A19" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D19" s="0"/>
+      <c r="E19" s="0"/>
+      <c r="F19" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="G19" s="0"/>
+      <c r="H19" s="0"/>
+      <c r="I19" s="14"/>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="F20" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="G20" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="H20" s="7"/>
+      <c r="A20" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="G20" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="15"/>
       <c r="I20" s="10" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="B21" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="C21" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="G21" s="12"/>
-      <c r="H21" s="11"/>
-      <c r="I21" s="14" t="s">
-        <v>37</v>
-      </c>
+      <c r="A21" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D21" s="15"/>
+      <c r="E21" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="F21" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="G21" s="15"/>
+      <c r="H21" s="15"/>
+      <c r="I21" s="10"/>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11"/>
-      <c r="B22" s="11"/>
-      <c r="C22" s="12"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="12"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="14"/>
+      <c r="A22" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G22" s="8"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="10"/>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>19</v>
-      </c>
+      <c r="A23" s="7"/>
+      <c r="B23" s="7"/>
+      <c r="C23" s="8"/>
       <c r="D23" s="9"/>
-      <c r="E23" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="G23" s="8" t="s">
-        <v>22</v>
-      </c>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="8"/>
       <c r="H23" s="7"/>
-      <c r="I23" s="10" t="s">
-        <v>39</v>
-      </c>
+      <c r="I23" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="B24" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="C24" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G24" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H24" s="7"/>
+      <c r="I24" s="10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="C25" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="G24" s="12"/>
-      <c r="H24" s="11"/>
-      <c r="I24" s="14" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7"/>
-      <c r="B25" s="7"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="8"/>
-      <c r="H25" s="7"/>
-      <c r="I25" s="15"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G25" s="12"/>
+      <c r="H25" s="11"/>
+      <c r="I25" s="14" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="11"/>
-      <c r="B26" s="11"/>
-      <c r="C26" s="12"/>
+      <c r="A26" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>19</v>
+      </c>
       <c r="D26" s="13"/>
-      <c r="E26" s="13"/>
-      <c r="F26" s="13"/>
+      <c r="E26" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="F26" s="13" t="s">
+        <v>21</v>
+      </c>
       <c r="G26" s="12"/>
       <c r="H26" s="11"/>
-      <c r="I26" s="14"/>
+      <c r="I26" s="14" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7"/>
-      <c r="B27" s="7"/>
-      <c r="C27" s="8"/>
+      <c r="A27" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>19</v>
+      </c>
       <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9"/>
+      <c r="E27" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>21</v>
+      </c>
       <c r="G27" s="8"/>
       <c r="H27" s="7"/>
-      <c r="I27" s="15"/>
+      <c r="I27" s="17" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="11"/>
-      <c r="B28" s="11"/>
-      <c r="C28" s="12"/>
+      <c r="A28" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>19</v>
+      </c>
       <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
-      <c r="F28" s="13"/>
+      <c r="E28" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="F28" s="13" t="s">
+        <v>21</v>
+      </c>
       <c r="G28" s="12"/>
       <c r="H28" s="11"/>
-      <c r="I28" s="14"/>
+      <c r="I28" s="18" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7"/>
-      <c r="B29" s="7"/>
-      <c r="C29" s="8"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="9"/>
-      <c r="F29" s="9"/>
-      <c r="G29" s="8"/>
-      <c r="H29" s="7"/>
-      <c r="I29" s="15"/>
+      <c r="A29" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B29" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D29" s="13"/>
+      <c r="E29" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="F29" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G29" s="12"/>
+      <c r="H29" s="11"/>
+      <c r="I29" s="18" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="11"/>
-      <c r="B30" s="11"/>
-      <c r="C30" s="12"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="13"/>
-      <c r="G30" s="12"/>
-      <c r="H30" s="11"/>
-      <c r="I30" s="14"/>
+      <c r="A30" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D30" s="9"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G30" s="8"/>
+      <c r="H30" s="7"/>
+      <c r="I30" s="10" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="7"/>
-      <c r="B31" s="7"/>
-      <c r="C31" s="8"/>
-      <c r="D31" s="9"/>
-      <c r="E31" s="9"/>
-      <c r="F31" s="9"/>
-      <c r="G31" s="8"/>
-      <c r="H31" s="7"/>
-      <c r="I31" s="15"/>
+      <c r="A31" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B31" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="C31" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
+      <c r="F31" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G31" s="12"/>
+      <c r="H31" s="11"/>
+      <c r="I31" s="14"/>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="11"/>
-      <c r="B32" s="11"/>
-      <c r="C32" s="12"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="13"/>
-      <c r="G32" s="12"/>
-      <c r="H32" s="11"/>
-      <c r="I32" s="14"/>
+      <c r="A32" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B32" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="C32" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D32" s="15"/>
+      <c r="E32" s="15"/>
+      <c r="F32" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="G32" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H32" s="15"/>
+      <c r="I32" s="10" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="7"/>
-      <c r="B33" s="7"/>
-      <c r="C33" s="8"/>
-      <c r="D33" s="9"/>
-      <c r="E33" s="9"/>
-      <c r="F33" s="9"/>
-      <c r="G33" s="8"/>
-      <c r="H33" s="7"/>
-      <c r="I33" s="15"/>
+      <c r="A33" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B33" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D33" s="0"/>
+      <c r="E33" s="0"/>
+      <c r="F33" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="G33" s="0"/>
+      <c r="H33" s="0"/>
+      <c r="I33" s="14"/>
     </row>
     <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="11"/>
-      <c r="B34" s="11"/>
-      <c r="C34" s="12"/>
-      <c r="D34" s="13"/>
-      <c r="E34" s="13"/>
-      <c r="F34" s="13"/>
-      <c r="G34" s="12"/>
-      <c r="H34" s="11"/>
-      <c r="I34" s="14"/>
+      <c r="A34" s="7"/>
+      <c r="B34" s="7"/>
+      <c r="C34" s="8"/>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="8"/>
+      <c r="H34" s="7"/>
+      <c r="I34" s="10"/>
     </row>
     <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="7"/>
-      <c r="B35" s="7"/>
-      <c r="C35" s="8"/>
-      <c r="D35" s="9"/>
-      <c r="E35" s="9"/>
-      <c r="F35" s="9"/>
-      <c r="G35" s="8"/>
-      <c r="H35" s="7"/>
-      <c r="I35" s="15"/>
+      <c r="A35" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B35" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D35" s="13"/>
+      <c r="E35" s="13"/>
+      <c r="F35" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G35" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="H35" s="11"/>
+      <c r="I35" s="14"/>
     </row>
     <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="11"/>
-      <c r="B36" s="11"/>
-      <c r="C36" s="12"/>
-      <c r="D36" s="13"/>
-      <c r="E36" s="13"/>
-      <c r="F36" s="13"/>
-      <c r="G36" s="12"/>
-      <c r="H36" s="11"/>
-      <c r="I36" s="14"/>
+      <c r="A36" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G36" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="H36" s="7"/>
+      <c r="I36" s="10"/>
     </row>
     <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="7"/>
-      <c r="B37" s="7"/>
-      <c r="C37" s="8"/>
-      <c r="D37" s="9"/>
-      <c r="E37" s="9"/>
-      <c r="F37" s="9"/>
-      <c r="G37" s="8"/>
-      <c r="H37" s="7"/>
-      <c r="I37" s="15"/>
+      <c r="A37" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B37" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C37" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D37" s="13"/>
+      <c r="E37" s="13"/>
+      <c r="F37" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G37" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H37" s="11"/>
+      <c r="I37" s="14"/>
     </row>
     <row r="38" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="11"/>
-      <c r="B38" s="11"/>
-      <c r="C38" s="12"/>
-      <c r="D38" s="13"/>
-      <c r="E38" s="13"/>
-      <c r="F38" s="13"/>
-      <c r="G38" s="12"/>
-      <c r="H38" s="11"/>
+      <c r="A38" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B38" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C38" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D38" s="0"/>
+      <c r="E38" s="0"/>
+      <c r="F38" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="G38" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="H38" s="0"/>
       <c r="I38" s="14"/>
     </row>
     <row r="39" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="7"/>
-      <c r="B39" s="7"/>
-      <c r="C39" s="8"/>
-      <c r="D39" s="9"/>
-      <c r="E39" s="9"/>
-      <c r="F39" s="9"/>
-      <c r="G39" s="8"/>
-      <c r="H39" s="7"/>
-      <c r="I39" s="15"/>
+      <c r="A39" s="11"/>
+      <c r="B39" s="11"/>
+      <c r="C39" s="12"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="13"/>
+      <c r="F39" s="13"/>
+      <c r="G39" s="12"/>
+      <c r="H39" s="11"/>
+      <c r="I39" s="14"/>
     </row>
     <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="11"/>
-      <c r="B40" s="11"/>
-      <c r="C40" s="12"/>
+      <c r="A40" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B40" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C40" s="12" t="s">
+        <v>19</v>
+      </c>
       <c r="D40" s="13"/>
       <c r="E40" s="13"/>
-      <c r="F40" s="13"/>
-      <c r="G40" s="12"/>
+      <c r="F40" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G40" s="12" t="s">
+        <v>22</v>
+      </c>
       <c r="H40" s="11"/>
-      <c r="I40" s="14"/>
+      <c r="I40" s="14" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="7"/>
-      <c r="B41" s="7"/>
-      <c r="C41" s="8"/>
+      <c r="A41" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>25</v>
+      </c>
       <c r="D41" s="9"/>
       <c r="E41" s="9"/>
-      <c r="F41" s="9"/>
-      <c r="G41" s="8"/>
+      <c r="F41" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G41" s="8" t="s">
+        <v>61</v>
+      </c>
       <c r="H41" s="7"/>
-      <c r="I41" s="15"/>
+      <c r="I41" s="10"/>
     </row>
     <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="11"/>
-      <c r="B42" s="11"/>
-      <c r="C42" s="12"/>
+      <c r="A42" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B42" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C42" s="12" t="s">
+        <v>19</v>
+      </c>
       <c r="D42" s="13"/>
       <c r="E42" s="13"/>
-      <c r="F42" s="13"/>
-      <c r="G42" s="12"/>
+      <c r="F42" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G42" s="15" t="n">
+        <v>1</v>
+      </c>
       <c r="H42" s="11"/>
       <c r="I42" s="14"/>
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="7"/>
-      <c r="B43" s="7"/>
-      <c r="C43" s="8"/>
-      <c r="D43" s="9"/>
-      <c r="E43" s="9"/>
-      <c r="F43" s="9"/>
-      <c r="G43" s="8"/>
-      <c r="H43" s="7"/>
-      <c r="I43" s="15"/>
+      <c r="A43" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B43" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C43" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D43" s="0"/>
+      <c r="E43" s="0"/>
+      <c r="F43" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="G43" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="H43" s="0"/>
+      <c r="I43" s="14"/>
     </row>
     <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="11"/>
-      <c r="B44" s="11"/>
-      <c r="C44" s="12"/>
-      <c r="D44" s="13"/>
-      <c r="E44" s="13"/>
-      <c r="F44" s="13"/>
-      <c r="G44" s="12"/>
-      <c r="H44" s="11"/>
-      <c r="I44" s="14"/>
+      <c r="A44" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B44" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C44" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D44" s="15"/>
+      <c r="E44" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="F44" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="G44" s="15"/>
+      <c r="H44" s="15"/>
+      <c r="I44" s="10"/>
     </row>
     <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="7"/>
-      <c r="B45" s="7"/>
-      <c r="C45" s="8"/>
+      <c r="A45" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B45" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C45" s="8" t="s">
+        <v>19</v>
+      </c>
       <c r="D45" s="9"/>
-      <c r="E45" s="9"/>
-      <c r="F45" s="9"/>
+      <c r="E45" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F45" s="9" t="s">
+        <v>21</v>
+      </c>
       <c r="G45" s="8"/>
       <c r="H45" s="7"/>
-      <c r="I45" s="15"/>
+      <c r="I45" s="10"/>
     </row>
     <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="11"/>
-      <c r="B46" s="11"/>
-      <c r="C46" s="12"/>
-      <c r="D46" s="13"/>
-      <c r="E46" s="13"/>
-      <c r="F46" s="13"/>
-      <c r="G46" s="12"/>
-      <c r="H46" s="11"/>
-      <c r="I46" s="14"/>
+      <c r="A46" s="7"/>
+      <c r="B46" s="7"/>
+      <c r="C46" s="8"/>
+      <c r="D46" s="9"/>
+      <c r="E46" s="9"/>
+      <c r="F46" s="9"/>
+      <c r="G46" s="8"/>
+      <c r="H46" s="7"/>
+      <c r="I46" s="10"/>
     </row>
     <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="7"/>
-      <c r="B47" s="7"/>
-      <c r="C47" s="8"/>
-      <c r="D47" s="9"/>
-      <c r="E47" s="9"/>
-      <c r="F47" s="9"/>
-      <c r="G47" s="8"/>
-      <c r="H47" s="7"/>
-      <c r="I47" s="15"/>
+      <c r="A47" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B47" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C47" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D47" s="13"/>
+      <c r="E47" s="13"/>
+      <c r="F47" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G47" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="H47" s="11"/>
+      <c r="I47" s="14" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="11"/>
-      <c r="B48" s="11"/>
-      <c r="C48" s="12"/>
-      <c r="D48" s="13"/>
-      <c r="E48" s="13"/>
-      <c r="F48" s="13"/>
-      <c r="G48" s="12"/>
-      <c r="H48" s="11"/>
-      <c r="I48" s="14"/>
+      <c r="A48" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B48" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="C48" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="D48" s="9"/>
+      <c r="E48" s="9"/>
+      <c r="F48" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G48" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="H48" s="7"/>
+      <c r="I48" s="10"/>
     </row>
     <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="7"/>
-      <c r="B49" s="7"/>
-      <c r="C49" s="8"/>
-      <c r="D49" s="9"/>
-      <c r="E49" s="9"/>
-      <c r="F49" s="9"/>
-      <c r="G49" s="8"/>
-      <c r="H49" s="7"/>
-      <c r="I49" s="15"/>
+      <c r="A49" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B49" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C49" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D49" s="13"/>
+      <c r="E49" s="13"/>
+      <c r="F49" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G49" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H49" s="11"/>
+      <c r="I49" s="14"/>
     </row>
     <row r="50" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="11"/>
-      <c r="B50" s="11"/>
-      <c r="C50" s="12"/>
-      <c r="D50" s="13"/>
-      <c r="E50" s="13"/>
-      <c r="F50" s="13"/>
-      <c r="G50" s="12"/>
-      <c r="H50" s="11"/>
+      <c r="A50" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B50" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C50" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D50" s="0"/>
+      <c r="E50" s="0"/>
+      <c r="F50" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="G50" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="H50" s="0"/>
       <c r="I50" s="14"/>
     </row>
     <row r="51" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="7"/>
-      <c r="B51" s="7"/>
-      <c r="C51" s="8"/>
-      <c r="D51" s="9"/>
-      <c r="E51" s="9"/>
-      <c r="F51" s="9"/>
-      <c r="G51" s="8"/>
-      <c r="H51" s="7"/>
-      <c r="I51" s="15"/>
+      <c r="A51" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B51" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C51" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D51" s="15"/>
+      <c r="E51" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="F51" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="G51" s="15"/>
+      <c r="H51" s="15"/>
+      <c r="I51" s="10"/>
     </row>
     <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="11"/>
-      <c r="B52" s="11"/>
-      <c r="C52" s="12"/>
-      <c r="D52" s="13"/>
-      <c r="E52" s="13"/>
-      <c r="F52" s="13"/>
-      <c r="G52" s="12"/>
-      <c r="H52" s="11"/>
-      <c r="I52" s="14"/>
+      <c r="A52" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B52" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C52" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D52" s="9"/>
+      <c r="E52" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F52" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G52" s="8"/>
+      <c r="H52" s="7"/>
+      <c r="I52" s="10"/>
     </row>
     <row r="53" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="7"/>
-      <c r="B53" s="7"/>
-      <c r="C53" s="8"/>
-      <c r="D53" s="9"/>
-      <c r="E53" s="9"/>
-      <c r="F53" s="9"/>
-      <c r="G53" s="8"/>
-      <c r="H53" s="7"/>
-      <c r="I53" s="15"/>
+      <c r="A53" s="11"/>
+      <c r="B53" s="11"/>
+      <c r="C53" s="12"/>
+      <c r="D53" s="13"/>
+      <c r="E53" s="13"/>
+      <c r="F53" s="13"/>
+      <c r="G53" s="12"/>
+      <c r="H53" s="11"/>
+      <c r="I53" s="14"/>
     </row>
     <row r="54" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="11"/>
-      <c r="B54" s="11"/>
-      <c r="C54" s="12"/>
+      <c r="A54" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="B54" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C54" s="12" t="s">
+        <v>19</v>
+      </c>
       <c r="D54" s="13"/>
       <c r="E54" s="13"/>
-      <c r="F54" s="13"/>
-      <c r="G54" s="12"/>
+      <c r="F54" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G54" s="12" t="s">
+        <v>22</v>
+      </c>
       <c r="H54" s="11"/>
-      <c r="I54" s="14"/>
+      <c r="I54" s="14" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="7"/>
-      <c r="B55" s="7"/>
-      <c r="C55" s="8"/>
+      <c r="A55" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="B55" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="C55" s="8" t="s">
+        <v>25</v>
+      </c>
       <c r="D55" s="9"/>
       <c r="E55" s="9"/>
-      <c r="F55" s="9"/>
-      <c r="G55" s="8"/>
+      <c r="F55" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G55" s="8" t="s">
+        <v>61</v>
+      </c>
       <c r="H55" s="7"/>
-      <c r="I55" s="15"/>
+      <c r="I55" s="10"/>
     </row>
     <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="11"/>
-      <c r="B56" s="11"/>
-      <c r="C56" s="12"/>
+      <c r="A56" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="B56" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C56" s="12" t="s">
+        <v>19</v>
+      </c>
       <c r="D56" s="13"/>
       <c r="E56" s="13"/>
-      <c r="F56" s="13"/>
-      <c r="G56" s="12"/>
+      <c r="F56" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G56" s="15" t="n">
+        <v>1</v>
+      </c>
       <c r="H56" s="11"/>
       <c r="I56" s="14"/>
     </row>
     <row r="57" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="7"/>
-      <c r="B57" s="7"/>
-      <c r="C57" s="8"/>
-      <c r="D57" s="9"/>
-      <c r="E57" s="9"/>
-      <c r="F57" s="9"/>
-      <c r="G57" s="8"/>
-      <c r="H57" s="7"/>
-      <c r="I57" s="15"/>
+      <c r="A57" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="B57" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C57" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D57" s="0"/>
+      <c r="E57" s="0"/>
+      <c r="F57" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="G57" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="H57" s="0"/>
+      <c r="I57" s="14"/>
     </row>
     <row r="58" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="11"/>
-      <c r="B58" s="11"/>
-      <c r="C58" s="12"/>
-      <c r="D58" s="13"/>
-      <c r="E58" s="13"/>
-      <c r="F58" s="13"/>
-      <c r="G58" s="12"/>
-      <c r="H58" s="11"/>
-      <c r="I58" s="14"/>
+      <c r="A58" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="B58" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C58" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D58" s="15"/>
+      <c r="E58" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="F58" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="G58" s="15"/>
+      <c r="H58" s="15"/>
+      <c r="I58" s="10"/>
     </row>
     <row r="59" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="7"/>
-      <c r="B59" s="7"/>
-      <c r="C59" s="8"/>
+      <c r="A59" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="B59" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C59" s="8" t="s">
+        <v>19</v>
+      </c>
       <c r="D59" s="9"/>
-      <c r="E59" s="9"/>
-      <c r="F59" s="9"/>
+      <c r="E59" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F59" s="9" t="s">
+        <v>21</v>
+      </c>
       <c r="G59" s="8"/>
       <c r="H59" s="7"/>
-      <c r="I59" s="15"/>
-    </row>
-    <row r="60" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="11"/>
-      <c r="B60" s="11"/>
-      <c r="C60" s="12"/>
-      <c r="D60" s="13"/>
-      <c r="E60" s="13"/>
-      <c r="F60" s="13"/>
-      <c r="G60" s="12"/>
-      <c r="H60" s="11"/>
-      <c r="I60" s="14"/>
-    </row>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="I59" s="10"/>
+    </row>
+    <row r="60" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="61" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="62" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="63" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C10:C13 C19:C60" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C10:C13 C15:C18 C22:C31 C34:C37 C39:C42 C45:C49 C52:C56 C59" type="list">
       <formula1>Validações!$A$1:$A$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E10:E13 E19:E60" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E10:E13 E15:E18 E22:E31 E34:E37 E39:E42 E45:E49 E52:E56 E59" type="list">
       <formula1>Validações!$B$1:$B$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F10:F13 F19:F60" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F10:F13 F15:F18 F22:F31 F34:F37 F39:F42 F45:F49 F52:F56 F59" type="list">
       <formula1>Validações!$C$1:$C$2</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1630,89 +2104,89 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>41</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>42</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="B4" s="19" t="s">
-        <v>44</v>
+      <c r="A4" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="B4" s="20" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="B5" s="19" t="s">
-        <v>46</v>
+      <c r="A5" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="B6" s="19" t="s">
-        <v>48</v>
+      <c r="A6" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="B7" s="19" t="s">
-        <v>50</v>
+      <c r="A7" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="B7" s="20" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="B8" s="19" t="s">
-        <v>52</v>
+      <c r="A8" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="B8" s="20" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
-        <v>53</v>
-      </c>
-      <c r="B9" s="19" t="s">
-        <v>54</v>
+      <c r="A9" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="B9" s="20" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
-        <v>55</v>
-      </c>
-      <c r="B10" s="19" t="s">
-        <v>56</v>
+      <c r="A10" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="B10" s="20" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="B11" s="19" t="s">
-        <v>58</v>
+      <c r="A11" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="B11" s="20" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="s">
-        <v>59</v>
-      </c>
-      <c r="B12" s="19" t="s">
-        <v>60</v>
+      <c r="A12" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="B12" s="20" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20" t="s">
-        <v>61</v>
+      <c r="A14" s="21" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1720,7 +2194,7 @@
         <v>8</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>62</v>
+        <v>91</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>10</v>
@@ -1735,10 +2209,10 @@
         <v>13</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>63</v>
+        <v>92</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>64</v>
+        <v>93</v>
       </c>
       <c r="I16" s="6" t="s">
         <v>16</v>
@@ -1746,16 +2220,16 @@
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>65</v>
+        <v>94</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>66</v>
+        <v>95</v>
       </c>
       <c r="C17" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>67</v>
+        <v>96</v>
       </c>
       <c r="E17" s="13" t="s">
         <v>20</v>
@@ -1764,131 +2238,131 @@
         <v>21</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>68</v>
+        <v>97</v>
       </c>
       <c r="H17" s="11" t="s">
-        <v>69</v>
+        <v>98</v>
       </c>
       <c r="I17" s="14" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>65</v>
+        <v>94</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>71</v>
+        <v>100</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>72</v>
+        <v>101</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>21</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>69</v>
+        <v>98</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>75</v>
+        <v>104</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>65</v>
+        <v>94</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>76</v>
+        <v>105</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>72</v>
+        <v>101</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>67</v>
+        <v>96</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="F19" s="13" t="s">
         <v>21</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>69</v>
+        <v>98</v>
       </c>
       <c r="H19" s="11" t="s">
-        <v>77</v>
+        <v>106</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>65</v>
+        <v>94</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>78</v>
+        <v>107</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>33</v>
+        <v>108</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>69</v>
+        <v>98</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>21</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>69</v>
+        <v>98</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>79</v>
+        <v>109</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>65</v>
+        <v>94</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>80</v>
+        <v>110</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>72</v>
+        <v>101</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>81</v>
+        <v>111</v>
       </c>
       <c r="G21" s="12" t="s">
-        <v>82</v>
+        <v>112</v>
       </c>
       <c r="H21" s="11" t="s">
-        <v>83</v>
+        <v>113</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>65</v>
+        <v>94</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>84</v>
+        <v>114</v>
       </c>
       <c r="C22" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>67</v>
+        <v>96</v>
       </c>
       <c r="E22" s="9" t="s">
         <v>28</v>
@@ -1897,27 +2371,27 @@
         <v>21</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>69</v>
+        <v>98</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="I22" s="15" t="s">
-        <v>86</v>
+        <v>115</v>
+      </c>
+      <c r="I22" s="10" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>87</v>
+        <v>117</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>84</v>
+        <v>114</v>
       </c>
       <c r="C23" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>67</v>
+        <v>96</v>
       </c>
       <c r="E23" s="13" t="s">
         <v>20</v>
@@ -1926,65 +2400,65 @@
         <v>21</v>
       </c>
       <c r="G23" s="12" t="s">
-        <v>68</v>
+        <v>97</v>
       </c>
       <c r="H23" s="11" t="s">
-        <v>69</v>
+        <v>98</v>
       </c>
       <c r="I23" s="14" t="s">
-        <v>88</v>
+        <v>118</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>87</v>
+        <v>117</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>89</v>
+        <v>119</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>72</v>
+        <v>101</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>21</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>69</v>
+        <v>98</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>91</v>
+        <v>121</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>87</v>
+        <v>117</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>92</v>
+        <v>122</v>
       </c>
       <c r="C25" s="12" t="s">
         <v>19</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>93</v>
+        <v>123</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="F25" s="13" t="s">
         <v>21</v>
       </c>
       <c r="G25" s="12" t="s">
-        <v>94</v>
+        <v>124</v>
       </c>
       <c r="H25" s="11" t="s">
-        <v>95</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -2014,12 +2488,12 @@
         <v>20</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>81</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>96</v>
+        <v>126</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>28</v>
@@ -2030,23 +2504,23 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>97</v>
+        <v>127</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>98</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>99</v>
+        <v>129</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>100</v>
+        <v>130</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2056,27 +2530,27 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>101</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>33</v>
+        <v>108</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>102</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>103</v>
+        <v>132</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>104</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adiciona coluna id_servico na tabela ordem_servico e cria triggers para atualização de valor total
</commit_message>
<xml_diff>
--- a/docs/modelo_dicionario_de_dados.xlsx
+++ b/docs/modelo_dicionario_de_dados.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="689" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="172">
   <si>
     <t xml:space="preserve">MODELO DE DICIONÁRIO DE DADOS</t>
   </si>
@@ -343,9 +343,6 @@
   </si>
   <si>
     <t xml:space="preserve">nome_peca</t>
-  </si>
-  <si>
-    <t xml:space="preserve">preco_compra</t>
   </si>
   <si>
     <t xml:space="preserve">preco_venda</t>
@@ -690,7 +687,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -765,34 +762,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -1052,7 +1021,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I1002"/>
+  <dimension ref="A1:I1048576"/>
   <sheetFormatPr defaultColWidth="14.43359375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
@@ -2370,1071 +2339,1029 @@
       <c r="I68" s="3"/>
     </row>
     <row r="69" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="19" t="s">
+      <c r="A69" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="B69" s="19" t="s">
+      <c r="B69" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C69" s="20" t="s">
+      <c r="C69" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D69" s="21" t="s">
+      <c r="D69" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E69" s="21" t="s">
+      <c r="E69" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F69" s="21" t="s">
+      <c r="F69" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="G69" s="20" t="s">
+      <c r="G69" s="9" t="s">
         <v>22</v>
       </c>
       <c r="H69" s="3"/>
       <c r="I69" s="3"/>
     </row>
     <row r="70" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="22" t="s">
+      <c r="A70" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="B70" s="22" t="s">
+      <c r="B70" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="C70" s="23" t="s">
+      <c r="C70" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D70" s="24" t="s">
+      <c r="D70" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="E70" s="24" t="s">
+      <c r="E70" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="F70" s="24" t="s">
+      <c r="F70" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="G70" s="23" t="s">
+      <c r="G70" s="13" t="s">
         <v>79</v>
       </c>
       <c r="H70" s="3"/>
       <c r="I70" s="3"/>
     </row>
     <row r="71" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="19" t="s">
+      <c r="A71" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="B71" s="19" t="s">
+      <c r="B71" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="C71" s="20" t="s">
+      <c r="C71" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D71" s="21" t="s">
+      <c r="D71" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E71" s="21" t="s">
+      <c r="E71" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="F71" s="21" t="s">
+      <c r="F71" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="G71" s="20" t="s">
+      <c r="G71" s="9" t="s">
         <v>79</v>
       </c>
       <c r="H71" s="3"/>
       <c r="I71" s="3"/>
     </row>
     <row r="72" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="22" t="s">
+      <c r="A72" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="B72" s="22" t="s">
+      <c r="B72" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="C72" s="23" t="s">
+      <c r="C72" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D72" s="24" t="s">
+      <c r="D72" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="E72" s="24" t="s">
+      <c r="E72" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="F72" s="24" t="s">
+      <c r="F72" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="G72" s="23" t="s">
+      <c r="G72" s="13" t="s">
         <v>79</v>
       </c>
       <c r="H72" s="3"/>
       <c r="I72" s="3"/>
     </row>
     <row r="73" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="19" t="s">
+      <c r="A73" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="B73" s="19" t="s">
+      <c r="B73" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="C73" s="20" t="s">
+      <c r="C73" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D73" s="21" t="s">
+      <c r="D73" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E73" s="21" t="s">
+      <c r="E73" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="F73" s="21" t="s">
+      <c r="F73" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="G73" s="20" t="s">
+      <c r="G73" s="9" t="s">
         <v>79</v>
       </c>
       <c r="H73" s="3"/>
       <c r="I73" s="3"/>
     </row>
     <row r="74" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="22" t="s">
+      <c r="A74" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="B74" s="22" t="s">
+      <c r="B74" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="C74" s="23" t="s">
+      <c r="C74" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D74" s="24" t="s">
+      <c r="D74" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="E74" s="24" t="s">
+      <c r="E74" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="F74" s="24" t="s">
+      <c r="F74" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="G74" s="23" t="s">
+      <c r="G74" s="13" t="s">
         <v>79</v>
       </c>
       <c r="H74" s="3"/>
       <c r="I74" s="3"/>
     </row>
     <row r="75" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="19" t="s">
+      <c r="A75" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="B75" s="19" t="s">
+      <c r="B75" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="C75" s="20" t="s">
+      <c r="C75" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D75" s="21" t="s">
+      <c r="D75" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E75" s="21" t="s">
+      <c r="E75" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="F75" s="21" t="s">
+      <c r="F75" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="G75" s="20" t="s">
+      <c r="G75" s="9" t="s">
         <v>87</v>
       </c>
       <c r="H75" s="3"/>
       <c r="I75" s="3"/>
     </row>
     <row r="76" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="22" t="s">
+      <c r="A76" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="B76" s="22" t="s">
+      <c r="B76" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="C76" s="23" t="s">
+      <c r="C76" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D76" s="24" t="s">
+      <c r="D76" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="E76" s="24" t="s">
+      <c r="E76" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="F76" s="24" t="s">
+      <c r="F76" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="G76" s="23" t="s">
+      <c r="G76" s="13" t="s">
         <v>79</v>
       </c>
       <c r="H76" s="3"/>
       <c r="I76" s="3"/>
     </row>
     <row r="77" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="19" t="s">
+      <c r="A77" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="B77" s="19" t="s">
+      <c r="B77" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="C77" s="20" t="s">
+      <c r="C77" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D77" s="21" t="s">
+      <c r="D77" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E77" s="21" t="s">
+      <c r="E77" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="F77" s="21" t="s">
+      <c r="F77" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="G77" s="20" t="s">
+      <c r="G77" s="9" t="s">
         <v>79</v>
       </c>
       <c r="H77" s="3"/>
       <c r="I77" s="3"/>
     </row>
     <row r="78" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A78" s="22" t="s">
+      <c r="A78" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="B78" s="22" t="s">
+      <c r="B78" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="C78" s="23" t="s">
+      <c r="C78" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D78" s="24" t="s">
+      <c r="D78" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="E78" s="24" t="s">
+      <c r="E78" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="F78" s="24" t="s">
+      <c r="F78" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="G78" s="23" t="s">
+      <c r="G78" s="13" t="s">
         <v>79</v>
       </c>
       <c r="H78" s="3"/>
       <c r="I78" s="3"/>
     </row>
     <row r="79" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="19" t="s">
+      <c r="A79" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="B79" s="19" t="s">
+      <c r="B79" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="C79" s="20" t="s">
+      <c r="C79" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D79" s="21" t="s">
+      <c r="D79" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E79" s="21" t="s">
+      <c r="E79" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="F79" s="21" t="s">
+      <c r="F79" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="G79" s="20" t="s">
+      <c r="G79" s="9" t="s">
         <v>79</v>
       </c>
       <c r="H79" s="3"/>
       <c r="I79" s="3"/>
     </row>
     <row r="80" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A80" s="22" t="s">
+      <c r="A80" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="B80" s="22" t="s">
+      <c r="B80" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="C80" s="23" t="s">
+      <c r="C80" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D80" s="24" t="s">
+      <c r="D80" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="E80" s="24" t="s">
+      <c r="E80" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="F80" s="24" t="s">
+      <c r="F80" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="G80" s="23" t="s">
+      <c r="G80" s="13" t="s">
         <v>79</v>
       </c>
       <c r="H80" s="3"/>
       <c r="I80" s="3"/>
     </row>
     <row r="81" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A81" s="19" t="s">
+      <c r="A81" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="B81" s="19" t="s">
+      <c r="B81" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="C81" s="20" t="s">
+      <c r="C81" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D81" s="21" t="s">
+      <c r="D81" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E81" s="21" t="s">
+      <c r="E81" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="F81" s="21" t="s">
+      <c r="F81" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="G81" s="20" t="s">
+      <c r="G81" s="9" t="s">
         <v>79</v>
       </c>
       <c r="H81" s="3"/>
       <c r="I81" s="3"/>
     </row>
     <row r="82" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A82" s="25"/>
-      <c r="B82" s="25"/>
-      <c r="C82" s="25"/>
-      <c r="D82" s="25"/>
-      <c r="E82" s="25"/>
-      <c r="F82" s="25"/>
-      <c r="G82" s="25"/>
       <c r="H82" s="3"/>
       <c r="I82" s="3"/>
     </row>
     <row r="83" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A83" s="19" t="s">
+      <c r="A83" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="B83" s="19" t="s">
+      <c r="B83" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C83" s="20" t="s">
+      <c r="C83" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D83" s="21" t="s">
+      <c r="D83" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E83" s="21" t="s">
+      <c r="E83" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F83" s="21" t="s">
+      <c r="F83" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="G83" s="20" t="s">
+      <c r="G83" s="9" t="s">
         <v>22</v>
       </c>
       <c r="H83" s="3"/>
       <c r="I83" s="3"/>
     </row>
     <row r="84" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A84" s="22" t="s">
+      <c r="A84" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="B84" s="22" t="s">
+      <c r="B84" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="C84" s="23" t="s">
+      <c r="C84" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D84" s="24" t="s">
+      <c r="D84" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="E84" s="24" t="s">
+      <c r="E84" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="F84" s="24" t="s">
+      <c r="F84" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="G84" s="23" t="s">
+      <c r="G84" s="13" t="s">
         <v>79</v>
       </c>
       <c r="H84" s="3"/>
       <c r="I84" s="3"/>
     </row>
     <row r="85" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A85" s="19" t="s">
+      <c r="A85" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="B85" s="19" t="s">
+      <c r="B85" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="C85" s="20" t="s">
+      <c r="C85" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D85" s="21" t="s">
+      <c r="D85" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E85" s="21" t="s">
+      <c r="E85" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="F85" s="21" t="s">
+      <c r="F85" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="G85" s="20" t="s">
+      <c r="G85" s="9" t="s">
         <v>79</v>
       </c>
       <c r="H85" s="3"/>
       <c r="I85" s="3"/>
     </row>
     <row r="86" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A86" s="22" t="s">
+      <c r="A86" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="B86" s="22" t="s">
+      <c r="B86" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="C86" s="23" t="s">
+      <c r="C86" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D86" s="24" t="s">
+      <c r="D86" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="E86" s="24" t="s">
+      <c r="E86" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="F86" s="24" t="s">
+      <c r="F86" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="G86" s="23" t="s">
+      <c r="G86" s="13" t="s">
         <v>79</v>
       </c>
       <c r="H86" s="3"/>
       <c r="I86" s="3"/>
     </row>
     <row r="87" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A87" s="19" t="s">
+      <c r="A87" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="B87" s="19" t="s">
+      <c r="B87" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="C87" s="20" t="s">
+      <c r="C87" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D87" s="21" t="s">
+      <c r="D87" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E87" s="21" t="s">
+      <c r="E87" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="F87" s="21" t="s">
+      <c r="F87" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="G87" s="20" t="s">
+      <c r="G87" s="9" t="s">
         <v>79</v>
       </c>
       <c r="H87" s="3"/>
       <c r="I87" s="3"/>
     </row>
     <row r="88" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A88" s="22" t="s">
+      <c r="A88" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="B88" s="22" t="s">
+      <c r="B88" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="C88" s="23" t="s">
+      <c r="C88" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D88" s="24" t="s">
+      <c r="D88" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="E88" s="24" t="s">
+      <c r="E88" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="F88" s="24" t="s">
+      <c r="F88" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="G88" s="23" t="s">
+      <c r="G88" s="13" t="s">
         <v>87</v>
       </c>
       <c r="H88" s="3"/>
       <c r="I88" s="3"/>
     </row>
     <row r="89" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A89" s="0"/>
-      <c r="B89" s="0"/>
-      <c r="C89" s="0"/>
-      <c r="D89" s="0"/>
-      <c r="E89" s="0"/>
-      <c r="F89" s="0"/>
-      <c r="G89" s="0"/>
       <c r="H89" s="3"/>
       <c r="I89" s="3"/>
     </row>
     <row r="90" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A90" s="19" t="s">
+      <c r="A90" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="B90" s="19" t="s">
+      <c r="B90" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C90" s="20" t="s">
+      <c r="C90" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D90" s="21" t="s">
+      <c r="D90" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E90" s="21" t="s">
+      <c r="E90" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F90" s="21" t="s">
+      <c r="F90" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="G90" s="20" t="s">
+      <c r="G90" s="9" t="s">
         <v>22</v>
       </c>
       <c r="H90" s="3"/>
       <c r="I90" s="3"/>
     </row>
     <row r="91" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A91" s="22" t="s">
+      <c r="A91" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="B91" s="22" t="s">
+      <c r="B91" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="C91" s="23" t="s">
+      <c r="C91" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D91" s="24" t="s">
+      <c r="D91" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="E91" s="24" t="s">
+      <c r="E91" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="F91" s="24" t="s">
+      <c r="F91" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="G91" s="23" t="s">
+      <c r="G91" s="13" t="s">
         <v>79</v>
       </c>
       <c r="H91" s="3"/>
       <c r="I91" s="3"/>
     </row>
     <row r="92" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A92" s="19" t="s">
+      <c r="A92" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="B92" s="19" t="s">
+      <c r="B92" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="C92" s="20" t="s">
+      <c r="C92" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D92" s="21" t="s">
+      <c r="D92" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E92" s="21" t="s">
+      <c r="E92" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="F92" s="21" t="s">
+      <c r="F92" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="G92" s="20" t="s">
+      <c r="G92" s="9" t="s">
         <v>79</v>
       </c>
       <c r="H92" s="3"/>
       <c r="I92" s="3"/>
     </row>
     <row r="93" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A93" s="22" t="s">
+      <c r="A93" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="B93" s="22" t="s">
+      <c r="B93" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="C93" s="23" t="s">
+      <c r="C93" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D93" s="24" t="s">
+      <c r="D93" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="E93" s="24" t="s">
+      <c r="E93" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="F93" s="24" t="s">
+      <c r="F93" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="G93" s="23" t="s">
+      <c r="G93" s="13" t="s">
         <v>79</v>
       </c>
       <c r="H93" s="3"/>
       <c r="I93" s="3"/>
     </row>
     <row r="94" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A94" s="19" t="s">
+      <c r="A94" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="B94" s="19" t="s">
+      <c r="B94" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="C94" s="20" t="s">
+      <c r="C94" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="D94" s="21" t="s">
+      <c r="D94" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E94" s="21" t="s">
+      <c r="E94" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="F94" s="21" t="s">
+      <c r="F94" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="G94" s="20" t="s">
+      <c r="G94" s="9" t="s">
         <v>79</v>
       </c>
       <c r="H94" s="3"/>
       <c r="I94" s="3"/>
     </row>
     <row r="95" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A95" s="22" t="s">
+      <c r="A95" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="B95" s="22" t="s">
+      <c r="B95" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="C95" s="23" t="s">
+      <c r="C95" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D95" s="24" t="s">
+      <c r="D95" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="E95" s="24" t="s">
+      <c r="E95" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="F95" s="24" t="s">
+      <c r="F95" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="G95" s="23" t="s">
+      <c r="G95" s="13" t="s">
         <v>79</v>
       </c>
       <c r="H95" s="3"/>
       <c r="I95" s="3"/>
     </row>
     <row r="96" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A96" s="19" t="s">
+      <c r="A96" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="B96" s="19" t="s">
+      <c r="B96" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="C96" s="20" t="s">
+      <c r="C96" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D96" s="21" t="s">
+      <c r="D96" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E96" s="21" t="s">
+      <c r="E96" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="F96" s="21" t="s">
+      <c r="F96" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="G96" s="20" t="s">
+      <c r="G96" s="9" t="s">
         <v>79</v>
       </c>
       <c r="H96" s="3"/>
       <c r="I96" s="3"/>
     </row>
     <row r="97" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A97" s="22" t="s">
+      <c r="A97" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="B97" s="22" t="s">
+      <c r="B97" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="C97" s="23" t="s">
+      <c r="C97" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D97" s="24" t="s">
+      <c r="D97" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="E97" s="24" t="s">
+      <c r="E97" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="F97" s="24" t="s">
+      <c r="F97" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="G97" s="23" t="s">
+      <c r="G97" s="13" t="s">
         <v>87</v>
       </c>
       <c r="H97" s="3"/>
       <c r="I97" s="3"/>
     </row>
     <row r="98" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A98" s="19" t="s">
+      <c r="A98" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="B98" s="19" t="s">
+      <c r="B98" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C98" s="20" t="s">
+      <c r="C98" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D98" s="21" t="s">
+      <c r="D98" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E98" s="21" t="s">
+      <c r="E98" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="F98" s="21" t="s">
+      <c r="F98" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="G98" s="20" t="n">
+      <c r="G98" s="9" t="n">
         <v>1</v>
       </c>
       <c r="H98" s="3"/>
       <c r="I98" s="3"/>
     </row>
     <row r="99" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A99" s="25"/>
-      <c r="B99" s="25"/>
-      <c r="C99" s="25"/>
-      <c r="D99" s="25"/>
-      <c r="E99" s="25"/>
-      <c r="F99" s="25"/>
-      <c r="G99" s="25"/>
       <c r="H99" s="3"/>
       <c r="I99" s="3"/>
     </row>
     <row r="100" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A100" s="19" t="s">
+      <c r="A100" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="B100" s="19" t="s">
+      <c r="B100" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C100" s="20" t="s">
+      <c r="C100" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D100" s="21" t="s">
+      <c r="D100" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E100" s="21" t="s">
+      <c r="E100" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F100" s="21" t="s">
+      <c r="F100" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="G100" s="20" t="s">
+      <c r="G100" s="9" t="s">
         <v>22</v>
       </c>
       <c r="H100" s="3"/>
       <c r="I100" s="3"/>
     </row>
     <row r="101" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A101" s="22" t="s">
+      <c r="A101" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="B101" s="22" t="s">
+      <c r="B101" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="C101" s="23" t="s">
+      <c r="C101" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="D101" s="24" t="s">
+      <c r="D101" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="E101" s="24" t="s">
+      <c r="E101" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="F101" s="24" t="s">
+      <c r="F101" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="G101" s="23" t="s">
+      <c r="G101" s="13" t="s">
         <v>79</v>
       </c>
       <c r="H101" s="3"/>
       <c r="I101" s="3"/>
     </row>
     <row r="102" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A102" s="19" t="s">
+      <c r="A102" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="B102" s="19" t="s">
+      <c r="B102" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="C102" s="20" t="s">
+      <c r="C102" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D102" s="21" t="s">
+      <c r="D102" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E102" s="21" t="s">
+      <c r="E102" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="F102" s="21" t="s">
+      <c r="F102" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="G102" s="20" t="s">
+      <c r="G102" s="9" t="s">
         <v>79</v>
       </c>
       <c r="H102" s="3"/>
       <c r="I102" s="3"/>
     </row>
     <row r="103" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A103" s="22" t="s">
+      <c r="A103" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="B103" s="22" t="s">
+      <c r="B103" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C103" s="23" t="s">
+      <c r="C103" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D103" s="24" t="s">
+      <c r="D103" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E103" s="24" t="s">
+      <c r="E103" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="F103" s="24" t="s">
+      <c r="F103" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="G103" s="23" t="s">
+      <c r="G103" s="9" t="s">
         <v>79</v>
       </c>
       <c r="H103" s="3"/>
       <c r="I103" s="3"/>
     </row>
     <row r="104" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A104" s="19" t="s">
+      <c r="A104" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="B104" s="19" t="s">
+      <c r="B104" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="C104" s="20" t="s">
+      <c r="C104" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D104" s="21" t="s">
+      <c r="D104" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="E104" s="21" t="s">
+      <c r="E104" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="F104" s="21" t="s">
+      <c r="F104" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="G104" s="20" t="s">
+      <c r="G104" s="13" t="s">
         <v>79</v>
       </c>
       <c r="H104" s="3"/>
       <c r="I104" s="3"/>
     </row>
     <row r="105" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A105" s="22" t="s">
+      <c r="A105" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="B105" s="22" t="s">
-        <v>109</v>
-      </c>
-      <c r="C105" s="23" t="s">
+      <c r="B105" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C105" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D105" s="24" t="s">
+      <c r="D105" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E105" s="24" t="s">
-        <v>86</v>
-      </c>
-      <c r="F105" s="24" t="s">
+      <c r="E105" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="F105" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="G105" s="23" t="s">
+      <c r="G105" s="9" t="s">
         <v>79</v>
       </c>
       <c r="H105" s="3"/>
       <c r="I105" s="3"/>
     </row>
     <row r="106" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A106" s="19" t="s">
+      <c r="A106" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="B106" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="C106" s="20" t="s">
+      <c r="B106" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C106" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D106" s="21" t="s">
+      <c r="D106" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="E106" s="21" t="s">
+      <c r="E106" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="F106" s="21" t="s">
+      <c r="F106" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="G106" s="20" t="s">
+      <c r="G106" s="13" t="s">
         <v>79</v>
       </c>
       <c r="H106" s="3"/>
       <c r="I106" s="3"/>
     </row>
     <row r="107" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A107" s="22" t="s">
+      <c r="A107" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="B107" s="22" t="s">
-        <v>43</v>
-      </c>
-      <c r="C107" s="23" t="s">
-        <v>19</v>
-      </c>
-      <c r="D107" s="24" t="s">
+      <c r="B107" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C107" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D107" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E107" s="24" t="s">
-        <v>28</v>
-      </c>
-      <c r="F107" s="24" t="s">
+      <c r="E107" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="F107" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="G107" s="23" t="s">
-        <v>79</v>
+      <c r="G107" s="9" t="s">
+        <v>87</v>
       </c>
       <c r="H107" s="3"/>
       <c r="I107" s="3"/>
     </row>
     <row r="108" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A108" s="19" t="s">
+      <c r="A108" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="B108" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="C108" s="20" t="s">
-        <v>25</v>
-      </c>
-      <c r="D108" s="21" t="s">
+      <c r="B108" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C108" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D108" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="E108" s="21" t="s">
+      <c r="E108" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="F108" s="21" t="s">
+      <c r="F108" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="G108" s="20" t="s">
-        <v>87</v>
+      <c r="G108" s="13" t="n">
+        <v>1</v>
       </c>
       <c r="H108" s="3"/>
       <c r="I108" s="3"/>
     </row>
     <row r="109" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A109" s="22" t="s">
-        <v>105</v>
-      </c>
-      <c r="B109" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="C109" s="23" t="s">
-        <v>19</v>
-      </c>
-      <c r="D109" s="24" t="s">
-        <v>79</v>
-      </c>
-      <c r="E109" s="24" t="s">
-        <v>86</v>
-      </c>
-      <c r="F109" s="24" t="s">
-        <v>21</v>
-      </c>
-      <c r="G109" s="23" t="n">
-        <v>1</v>
-      </c>
       <c r="H109" s="3"/>
       <c r="I109" s="3"/>
     </row>
     <row r="110" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A110" s="25"/>
-      <c r="B110" s="25"/>
-      <c r="C110" s="25"/>
-      <c r="D110" s="25"/>
-      <c r="E110" s="25"/>
-      <c r="F110" s="25"/>
-      <c r="G110" s="25"/>
+      <c r="A110" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B110" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C110" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D110" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="E110" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F110" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G110" s="9" t="s">
+        <v>22</v>
+      </c>
       <c r="H110" s="3"/>
       <c r="I110" s="3"/>
     </row>
     <row r="111" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A111" s="19" t="s">
+      <c r="A111" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="B111" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="B111" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="C111" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="D111" s="21" t="s">
+      <c r="C111" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D111" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="E111" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="F111" s="21" t="s">
+      <c r="E111" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="F111" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="G111" s="20" t="s">
-        <v>22</v>
+      <c r="G111" s="13" t="s">
+        <v>79</v>
       </c>
       <c r="H111" s="3"/>
       <c r="I111" s="3"/>
     </row>
     <row r="112" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A112" s="22" t="s">
-        <v>110</v>
-      </c>
-      <c r="B112" s="22" t="s">
-        <v>111</v>
-      </c>
-      <c r="C112" s="23" t="s">
-        <v>25</v>
-      </c>
-      <c r="D112" s="24" t="s">
+      <c r="A112" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B112" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C112" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D112" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E112" s="24" t="s">
+      <c r="E112" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="F112" s="24" t="s">
+      <c r="F112" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="G112" s="23" t="s">
-        <v>79</v>
+      <c r="G112" s="9" t="n">
+        <v>1</v>
       </c>
       <c r="H112" s="3"/>
       <c r="I112" s="3"/>
     </row>
     <row r="113" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A113" s="19" t="s">
-        <v>110</v>
-      </c>
-      <c r="B113" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="C113" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="D113" s="21" t="s">
-        <v>79</v>
-      </c>
-      <c r="E113" s="21" t="s">
-        <v>86</v>
-      </c>
-      <c r="F113" s="21" t="s">
-        <v>21</v>
-      </c>
-      <c r="G113" s="20" t="n">
-        <v>1</v>
-      </c>
+      <c r="A113" s="3"/>
+      <c r="B113" s="3"/>
+      <c r="C113" s="3"/>
+      <c r="D113" s="3"/>
+      <c r="E113" s="3"/>
+      <c r="F113" s="3"/>
+      <c r="G113" s="3"/>
       <c r="H113" s="3"/>
       <c r="I113" s="3"/>
     </row>
@@ -13206,20 +13133,10 @@
       <c r="H1001" s="3"/>
       <c r="I1001" s="3"/>
     </row>
-    <row r="1002" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1002" s="3"/>
-      <c r="B1002" s="3"/>
-      <c r="C1002" s="3"/>
-      <c r="D1002" s="3"/>
-      <c r="E1002" s="3"/>
-      <c r="F1002" s="3"/>
-      <c r="G1002" s="3"/>
-      <c r="H1002" s="3"/>
-      <c r="I1002" s="3"/>
-    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F10:F13 F15:F18 F22:F33 F36:F39 F41:F44 F47:F51 F54:F58 F61 F69:F88 F90:F113" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F10:F13 F15:F18 F22:F33 F36:F39 F41:F44 F47:F51 F54:F58 F61 F69:F88 F90:F112" type="list">
       <formula1>Validações!$C$1:$C$2</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -13227,11 +13144,11 @@
       <formula1>Validações!$A$1:$A$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E10:E13 E15:E18 E22:E33 E36:E39 E41:E44 E47:E51 E54:E58 E61 E69:E88 E90:E113" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E10:E13 E15:E18 E22:E33 E36:E39 E41:E44 E47:E51 E54:E58 E61 E69:E88 E90:E112" type="list">
       <formula1>Validações!$B$1:$B$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C69:C88 C90:C113" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C69:C88 C90:C112" type="list">
       <formula1>Validações!$A$1:$A$12</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -13267,7 +13184,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -13280,7 +13197,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -13303,11 +13220,11 @@
       <c r="I3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="26" t="s">
+      <c r="A4" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>114</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>115</v>
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
@@ -13318,11 +13235,11 @@
       <c r="I4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="26" t="s">
+      <c r="A5" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>116</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>117</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
@@ -13333,11 +13250,11 @@
       <c r="I5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="26" t="s">
+      <c r="A6" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>118</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>119</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
@@ -13348,11 +13265,11 @@
       <c r="I6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="26" t="s">
+      <c r="A7" s="19" t="s">
+        <v>119</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>120</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>121</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
@@ -13363,11 +13280,11 @@
       <c r="I7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="26" t="s">
+      <c r="A8" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>122</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>123</v>
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
@@ -13378,11 +13295,11 @@
       <c r="I8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="26" t="s">
+      <c r="A9" s="19" t="s">
+        <v>123</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>124</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>125</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
@@ -13393,11 +13310,11 @@
       <c r="I9" s="3"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="26" t="s">
+      <c r="A10" s="19" t="s">
+        <v>125</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>126</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>127</v>
       </c>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
@@ -13408,11 +13325,11 @@
       <c r="I10" s="3"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="26" t="s">
+      <c r="A11" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>128</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>129</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
@@ -13423,11 +13340,11 @@
       <c r="I11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="26" t="s">
+      <c r="A12" s="19" t="s">
+        <v>129</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>130</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>131</v>
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
@@ -13449,8 +13366,8 @@
       <c r="I13" s="3"/>
     </row>
     <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="27" t="s">
-        <v>132</v>
+      <c r="A14" s="20" t="s">
+        <v>131</v>
       </c>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -13477,7 +13394,7 @@
         <v>8</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>10</v>
@@ -13492,10 +13409,10 @@
         <v>13</v>
       </c>
       <c r="G16" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="H16" s="7" t="s">
         <v>134</v>
-      </c>
-      <c r="H16" s="7" t="s">
-        <v>135</v>
       </c>
       <c r="I16" s="7" t="s">
         <v>16</v>
@@ -13503,16 +13420,16 @@
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="B17" s="12" t="s">
         <v>136</v>
-      </c>
-      <c r="B17" s="12" t="s">
-        <v>137</v>
       </c>
       <c r="C17" s="13" t="s">
         <v>19</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E17" s="14" t="s">
         <v>20</v>
@@ -13521,27 +13438,27 @@
         <v>21</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H17" s="12" t="s">
         <v>79</v>
       </c>
       <c r="I17" s="15" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B18" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="C18" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="D18" s="10" t="s">
         <v>142</v>
-      </c>
-      <c r="D18" s="10" t="s">
-        <v>143</v>
       </c>
       <c r="E18" s="10" t="s">
         <v>86</v>
@@ -13553,22 +13470,22 @@
         <v>79</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I18" s="3"/>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E19" s="14" t="s">
         <v>86</v>
@@ -13580,19 +13497,19 @@
         <v>79</v>
       </c>
       <c r="H19" s="12" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I19" s="3"/>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B20" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C20" s="9" t="s">
         <v>147</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>148</v>
       </c>
       <c r="D20" s="10" t="s">
         <v>79</v>
@@ -13607,22 +13524,22 @@
         <v>79</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="I20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C21" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="D21" s="14" t="s">
         <v>142</v>
-      </c>
-      <c r="D21" s="14" t="s">
-        <v>143</v>
       </c>
       <c r="E21" s="14" t="s">
         <v>86</v>
@@ -13631,25 +13548,25 @@
         <v>89</v>
       </c>
       <c r="G21" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="H21" s="12" t="s">
         <v>151</v>
-      </c>
-      <c r="H21" s="12" t="s">
-        <v>152</v>
       </c>
       <c r="I21" s="3"/>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>19</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E22" s="10" t="s">
         <v>28</v>
@@ -13661,24 +13578,24 @@
         <v>79</v>
       </c>
       <c r="H22" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="I22" s="11" t="s">
         <v>154</v>
-      </c>
-      <c r="I22" s="11" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C23" s="13" t="s">
         <v>19</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E23" s="14" t="s">
         <v>20</v>
@@ -13687,27 +13604,27 @@
         <v>21</v>
       </c>
       <c r="G23" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H23" s="12" t="s">
         <v>79</v>
       </c>
       <c r="I23" s="15" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B24" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="D24" s="10" t="s">
         <v>158</v>
-      </c>
-      <c r="C24" s="9" t="s">
-        <v>142</v>
-      </c>
-      <c r="D24" s="10" t="s">
-        <v>159</v>
       </c>
       <c r="E24" s="10" t="s">
         <v>86</v>
@@ -13719,22 +13636,22 @@
         <v>79</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I24" s="3"/>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C25" s="13" t="s">
         <v>19</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E25" s="14" t="s">
         <v>86</v>
@@ -13743,10 +13660,10 @@
         <v>21</v>
       </c>
       <c r="G25" s="13" t="s">
+        <v>162</v>
+      </c>
+      <c r="H25" s="12" t="s">
         <v>163</v>
-      </c>
-      <c r="H25" s="12" t="s">
-        <v>164</v>
       </c>
       <c r="I25" s="3"/>
     </row>
@@ -24510,7 +24427,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>28</v>
@@ -24521,15 +24438,15 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>166</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>86</v>
@@ -24537,7 +24454,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24547,12 +24464,12 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24562,12 +24479,12 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>